<commit_message>
Sync BD docs 2026-07-08-v1 (202607160246) from my-cloud-project@1ef608b
</commit_message>
<xml_diff>
--- a/Coiling_Bolts_Blood_Mage_BD指南.xlsx
+++ b/Coiling_Bolts_Blood_Mage_BD指南.xlsx
@@ -304,9 +304,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>2</col>
+      <col>1</col>
       <colOff>0</colOff>
-      <row>6</row>
+      <row>14</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -329,9 +329,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>3</col>
+      <col>2</col>
       <colOff>0</colOff>
-      <row>6</row>
+      <row>17</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -354,9 +354,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>3</col>
       <colOff>0</colOff>
-      <row>6</row>
+      <row>17</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -379,9 +379,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>4</col>
       <colOff>0</colOff>
-      <row>11</row>
+      <row>17</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -404,9 +404,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>1</col>
       <colOff>0</colOff>
-      <row>11</row>
+      <row>20</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -431,7 +431,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>14</row>
+      <row>25</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -456,7 +456,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>17</row>
+      <row>28</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -479,9 +479,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>2</col>
+      <col>1</col>
       <colOff>0</colOff>
-      <row>17</row>
+      <row>31</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -504,181 +504,6 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>3</col>
-      <colOff>0</colOff>
-      <row>17</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="10" name="Image 10" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId10"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>0</colOff>
-      <row>17</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="11" name="Image 11" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId11"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>20</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="12" name="Image 12" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId12"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>20</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="13" name="Image 13" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId13"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>25</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="14" name="Image 14" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId14"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>28</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="15" name="Image 15" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId15"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>31</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="16" name="Image 16" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId16"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
       <col>1</col>
       <colOff>0</colOff>
       <row>36</row>
@@ -687,11 +512,11 @@
     <ext cx="200025" cy="609600"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPr id="10" name="Image 10" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId17"/>
+        <a:blip cstate="print" r:embed="rId10"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -712,36 +537,11 @@
     <ext cx="609600" cy="609600"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="18" name="Image 18" descr="Picture"/>
+        <cNvPr id="11" name="Image 11" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId18"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>71</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="19" name="Image 19" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId19"/>
+        <a:blip cstate="print" r:embed="rId11"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2038,20 +1838,17 @@
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>細思施法
-(Considered Casting)</t>
+          <t>Considered Casting</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>混沌專精
-(Chaos Mastery)</t>
+          <t>Chaos Mastery</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>極盛 II
-(Zenith II)</t>
+          <t>Zenith II</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
@@ -2082,22 +1879,17 @@
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>★ 被輔助法術技能的施放速度減少15%
-★ 被輔助的法術造成35%更多傷害
-▶ 寂缠弹：施法速度换更多伤害</t>
+          <t>▶ 寂缠弹：施法速度换更多伤害</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>★ +1被輔助混沌技能寶石的等級
-▶ 混沌伤害辅助</t>
+          <t>▶ 混沌伤害辅助</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>★ 被輔助的技能增加25%魔力消耗效率
-★ 你的魔力高於最大魔力的90%時，被輔助的法術造成30%更多傷害
-▶ 零魔力技能可满层 Zenith</t>
+          <t>▶ 零魔力技能可满层 Zenith</t>
         </is>
       </c>
       <c r="F7" s="11" t="inlineStr">
@@ -2145,8 +1937,7 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>生命痕跡
-(Level)
+          <t>Life Remnants
 Lv.20</t>
         </is>
       </c>
@@ -2162,23 +1953,15 @@
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>卡塔爾的恢復
-(Date)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" outlineLevel="1" ht="124" customHeight="1">
+          <t>Khatal's Rejuvenation</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" outlineLevel="1" ht="36" customHeight="1">
       <c r="A12" s="10" t="n"/>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>★ 痕跡持續8秒
-★ 擊殺一名敵人時有25%機率生成一個痕跡
-★ 擊中敵人時產生1個痕跡，每3秒只能產生一個
-★ 每個痕跡賦予(11—410)生命
-★ base deal no damage 1
-★ base deal no damage over time 1
-★ skill desired amount override 1
-▶ 血法师赋予：生命痕跡回复</t>
+          <t>▶ 血法师赋予：生命痕跡回复</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
@@ -2193,9 +1976,7 @@
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>★ 被輔助技能所創造的痕跡會在拾取時賦予卡塔爾的回春
-★ base_cooldown_speed_+%
-▶ 生命痕跡族裔辅助</t>
+          <t>▶ 生命痕跡族裔辅助</t>
         </is>
       </c>
     </row>
@@ -2280,8 +2061,7 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>瀆神
-(Level)
+          <t>Blasphemy
 Lv.19</t>
         </is>
       </c>
@@ -2318,16 +2098,7 @@
       <c r="A18" s="10" t="n"/>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>■ 移除玩家極地裝甲、暴風之盾、鮮血狂怒、熔岩護盾、迷蹤、石化之血、光環、病疫之難、凋零之步、詛咒和捷光環的視覺特效。
-■ 你的光環特效替換為力場防護罩。
-■ 你的光環特效替換為一個閃耀著電光的骷髏。
-■ 你的光環特效替還為一個被地獄之火圍繞的骷髏。
-★ 插槽中的詛咒技能會以光環的形式影響周圍
-★ 每個插槽中的詛咒占用60精魂
-★ 被輔助的詛咒有(41—50)%更少效果幅度
-★ 插槽中的技能在基礎範圍上額外增加+1公尺
-★ base deal no damage 1
-▶ 诅咒光环</t>
+          <t>▶ 诅咒光环</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
@@ -2405,8 +2176,7 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>混沌專精
-(Chaos Mastery)</t>
+          <t>Chaos Mastery</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
@@ -2427,8 +2197,7 @@
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>★ +1被輔助混沌技能寶石的等級
-▶ 混沌伤害辅助</t>
+          <t>▶ 混沌伤害辅助</t>
         </is>
       </c>
       <c r="D21" s="11" t="inlineStr">
@@ -3037,27 +2806,17 @@
       </c>
       <c r="B71" s="12" t="inlineStr">
         <is>
-          <t>殘酷塑像
-(Effigy of Cruelty)</t>
+          <t>Effigy of Cruelty</t>
         </is>
       </c>
       <c r="C71" s="13" t="n"/>
     </row>
-    <row r="72" outlineLevel="1" ht="204" customHeight="1">
+    <row r="72" outlineLevel="1" ht="72" customHeight="1">
       <c r="A72" s="10" t="n"/>
       <c r="B72" s="11" t="inlineStr"/>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>殘酷塑像 (Effigy of Cruelty)
-底材：Antler Focus
-需求:  等級 10, 17 智慧
-★ +(20—30)最大能量護盾
-★ 增加(40—50)%法術傷害
-★ +10點智慧
-★ +(7—13)%混沌抗性
-★ 以法術暴擊時，施加(1—3)層的暴擊弱點
-「The horrors we imagined as children
-still exist somewhere in the dark...」
+          <t>Effigy of Cruelty
 ▶ BD 用途：II 组副手：法术暴击叠 Critical Weakness
 🔗 https://poe2db.tw/tw/Effigy_of_Cruelty
 ▶ Entangle 叠 Critical Weakness（冷/混沌变体可选 The Wicked Quill）</t>

</xml_diff>

<commit_message>
Sync BD docs 2026-07-08-v1 (202607160248) from my-cloud-project@7b30e9e
</commit_message>
<xml_diff>
--- a/Coiling_Bolts_Blood_Mage_BD指南.xlsx
+++ b/Coiling_Bolts_Blood_Mage_BD指南.xlsx
@@ -279,7 +279,7 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>3</col>
       <colOff>0</colOff>
       <row>6</row>
       <rowOff>0</rowOff>
@@ -304,9 +304,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>4</col>
       <colOff>0</colOff>
-      <row>14</row>
+      <row>6</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -329,9 +329,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>2</col>
+      <col>1</col>
       <colOff>0</colOff>
-      <row>17</row>
+      <row>11</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -354,9 +354,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>3</col>
+      <col>4</col>
       <colOff>0</colOff>
-      <row>17</row>
+      <row>11</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -379,9 +379,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>1</col>
       <colOff>0</colOff>
-      <row>17</row>
+      <row>14</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -406,7 +406,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>20</row>
+      <row>17</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -429,9 +429,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>2</col>
       <colOff>0</colOff>
-      <row>25</row>
+      <row>17</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -454,9 +454,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>3</col>
       <colOff>0</colOff>
-      <row>28</row>
+      <row>17</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -479,9 +479,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>4</col>
       <colOff>0</colOff>
-      <row>31</row>
+      <row>17</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -506,10 +506,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>36</row>
+      <row>20</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="200025" cy="609600"/>
+    <ext cx="609600" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="10" name="Image 10" descr="Picture"/>
@@ -529,9 +529,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>2</col>
       <colOff>0</colOff>
-      <row>39</row>
+      <row>20</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -542,6 +542,81 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>28</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="13" name="Image 13" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>31</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="14" name="Image 14" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId14"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1831,8 +1906,7 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>寂纏彈
-(Level)
+          <t>Coiling Bolts
 Lv.20</t>
         </is>
       </c>
@@ -1843,12 +1917,14 @@
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>Chaos Mastery</t>
+          <t>混沌專精
+(Chaos Mastery)</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>Zenith II</t>
+          <t>極盛 II
+(Zenith II)</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
@@ -1862,19 +1938,11 @@
         </is>
       </c>
     </row>
-    <row r="7" outlineLevel="1" ht="132" customHeight="1">
+    <row r="7" outlineLevel="1" ht="84" customHeight="1">
       <c r="A7" s="10" t="n"/>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>★ 造成(9—279)至(14—418)物理傷害
-★ 投射物數量詞綴套用至投射物裂化目標數量
-★ 投射物會朝2個目標分裂
-★ 可從任意數量的受詛咒目標連鎖
-★ 增加50%連鎖範圍
-★ 造成(8—244)至(15—453)混沌傷害
-★ base is projectile 1
-★ can perform skill while moving 1
-▶ 主输出：物理+混沌双投射物，分裂+无限连锁受诅咒目标</t>
+          <t>▶ 主输出：物理+混沌双投射物，分裂+无限连锁受诅咒目标</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
@@ -1884,12 +1952,15 @@
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>▶ 混沌伤害辅助</t>
+          <t>★ +1被輔助混沌技能寶石的等級
+▶ 混沌伤害辅助</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>▶ 零魔力技能可满层 Zenith</t>
+          <t>★ 被輔助的技能增加25%魔力消耗效率
+★ 你的魔力高於最大魔力的90%時，被輔助的法術造成30%更多傷害
+▶ 零魔力技能可满层 Zenith</t>
         </is>
       </c>
       <c r="F7" s="11" t="inlineStr">
@@ -1937,7 +2008,8 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Life Remnants
+          <t>生命痕跡
+(Level)
 Lv.20</t>
         </is>
       </c>
@@ -1953,15 +2025,23 @@
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>Khatal's Rejuvenation</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" outlineLevel="1" ht="36" customHeight="1">
+          <t>卡塔爾的恢復
+(Date)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" outlineLevel="1" ht="124" customHeight="1">
       <c r="A12" s="10" t="n"/>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>▶ 血法师赋予：生命痕跡回复</t>
+          <t>★ 痕跡持續8秒
+★ 擊殺一名敵人時有25%機率生成一個痕跡
+★ 擊中敵人時產生1個痕跡，每3秒只能產生一個
+★ 每個痕跡賦予(11—410)生命
+★ base deal no damage 1
+★ base deal no damage over time 1
+★ skill desired amount override 1
+▶ 血法师赋予：生命痕跡回复</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
@@ -1976,7 +2056,9 @@
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>▶ 生命痕跡族裔辅助</t>
+          <t>★ 被輔助技能所創造的痕跡會在拾取時賦予卡塔爾的回春
+★ base_cooldown_speed_+%
+▶ 生命痕跡族裔辅助</t>
         </is>
       </c>
     </row>
@@ -2061,7 +2143,8 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>Blasphemy
+          <t>瀆神
+(Level)
 Lv.19</t>
         </is>
       </c>
@@ -2098,7 +2181,16 @@
       <c r="A18" s="10" t="n"/>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>▶ 诅咒光环</t>
+          <t>■ 移除玩家極地裝甲、暴風之盾、鮮血狂怒、熔岩護盾、迷蹤、石化之血、光環、病疫之難、凋零之步、詛咒和捷光環的視覺特效。
+■ 你的光環特效替換為力場防護罩。
+■ 你的光環特效替換為一個閃耀著電光的骷髏。
+■ 你的光環特效替還為一個被地獄之火圍繞的骷髏。
+★ 插槽中的詛咒技能會以光環的形式影響周圍
+★ 每個插槽中的詛咒占用60精魂
+★ 被輔助的詛咒有(41—50)%更少效果幅度
+★ 插槽中的技能在基礎範圍上額外增加+1公尺
+★ base deal no damage 1
+▶ 诅咒光环</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
@@ -2176,7 +2268,8 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>Chaos Mastery</t>
+          <t>混沌專精
+(Chaos Mastery)</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
@@ -2197,7 +2290,8 @@
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>▶ 混沌伤害辅助</t>
+          <t>★ +1被輔助混沌技能寶石的等級
+▶ 混沌伤害辅助</t>
         </is>
       </c>
       <c r="D21" s="11" t="inlineStr">
@@ -2490,31 +2584,17 @@
       </c>
       <c r="B36" s="12" t="inlineStr">
         <is>
-          <t>臨界纏繞
-(Liminal Coil)</t>
+          <t>Liminal Coil</t>
         </is>
       </c>
       <c r="C36" s="13" t="n"/>
     </row>
-    <row r="37" outlineLevel="1" ht="264" customHeight="1">
+    <row r="37" outlineLevel="1" ht="72" customHeight="1">
       <c r="A37" s="10" t="n"/>
       <c r="B37" s="11" t="inlineStr"/>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>臨界纏繞 (Liminal Coil)
-底材：Twisted Wand
-需求:  等級 65, 114 智慧
-■ 賦予技能: 寂纏彈
-★ 增加(71—113)%法術傷害
-★ 增加(7—13)%施放速度
-★ 你施加的詛咒幅度為零
-★ 你施加的詛咒無視詛咒上限
-★ 目標每受一個詛咒影響，法術擊中即獲得(23—31)%傷害的額外混沌傷害
-★ 目標每受一個詛咒影響，法術擊中即獲得(23—31)%傷害的額外物理傷害
-「In that moment, Viridi's bones became 
-branches, weaving over the Darkness. 
-She coiled around the nothing, 
-trapping it within her everything.」
+          <t>Liminal Coil
 ▶ BD 用途：BD 核心：赋予寂缠弹；诅咒幅度归零但无视诅咒上限，每诅咒巨额额外物理/混沌
 🔗 https://poe2db.tw/tw/Liminal_Coil
 ▶ 唯一来源寂缠弹；6 诅咒各 +25~31% 额外物理/混沌</t>
@@ -2530,27 +2610,17 @@
       </c>
       <c r="B39" s="12" t="inlineStr">
         <is>
-          <t>極地之嗥
-(Alpha's Howl)</t>
+          <t>Alpha's Howl</t>
         </is>
       </c>
       <c r="C39" s="13" t="n"/>
     </row>
-    <row r="40" outlineLevel="1" ht="204" customHeight="1">
+    <row r="40" outlineLevel="1" ht="72" customHeight="1">
       <c r="A40" s="10" t="n"/>
       <c r="B40" s="11" t="inlineStr"/>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>極地之嗥 (Alpha's Howl)
-底材：Armoured Cap
-需求:  等級 65, 91 敏捷
-★ 增加(80—100)%閃避值
-★ +100精魂
-★ +(50—75)%冰冷抗性
-★ 存在範圍的範圍加倍
-「Nature respects the strong
-And paints the snow red
-With the blood of the weak」
+          <t>Alpha's Howl
 ▶ BD 用途：+100 Spirit，Blasphemy 多诅咒必备
 🔗 https://poe2db.tw/tw/Alphas_Howl
 ▶ +100 Spirit，Blasphemy 必备</t>

</xml_diff>

<commit_message>
Sync BD docs 2026-07-08-v1 (202607160255) from my-cloud-project@8c157a3
</commit_message>
<xml_diff>
--- a/Coiling_Bolts_Blood_Mage_BD指南.xlsx
+++ b/Coiling_Bolts_Blood_Mage_BD指南.xlsx
@@ -279,7 +279,7 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>3</col>
+      <col>1</col>
       <colOff>0</colOff>
       <row>6</row>
       <rowOff>0</rowOff>
@@ -304,7 +304,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>2</col>
       <colOff>0</colOff>
       <row>6</row>
       <rowOff>0</rowOff>
@@ -329,9 +329,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>3</col>
       <colOff>0</colOff>
-      <row>11</row>
+      <row>6</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -356,7 +356,7 @@
     <from>
       <col>4</col>
       <colOff>0</colOff>
-      <row>11</row>
+      <row>6</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -379,9 +379,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>4</col>
       <colOff>0</colOff>
-      <row>14</row>
+      <row>11</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -406,7 +406,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>17</row>
+      <row>14</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -429,7 +429,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>2</col>
+      <col>1</col>
       <colOff>0</colOff>
       <row>17</row>
       <rowOff>0</rowOff>
@@ -454,7 +454,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>3</col>
+      <col>2</col>
       <colOff>0</colOff>
       <row>17</row>
       <rowOff>0</rowOff>
@@ -479,7 +479,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>3</col>
       <colOff>0</colOff>
       <row>17</row>
       <rowOff>0</rowOff>
@@ -504,7 +504,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>2</col>
       <colOff>0</colOff>
       <row>20</row>
       <rowOff>0</rowOff>
@@ -529,9 +529,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>2</col>
+      <col>1</col>
       <colOff>0</colOff>
-      <row>20</row>
+      <row>25</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -556,7 +556,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>25</row>
+      <row>28</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -581,10 +581,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>28</row>
+      <row>36</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="609600" cy="609600"/>
+    <ext cx="200025" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="13" name="Image 13" descr="Picture"/>
@@ -606,7 +606,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>31</row>
+      <row>39</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -617,6 +617,31 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId14"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>71</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId15"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1906,13 +1931,15 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Coiling Bolts
+          <t>寂纏彈
+(Level)
 Lv.20</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Considered Casting</t>
+          <t>細思施法
+(Considered Casting)</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
@@ -1938,16 +1965,26 @@
         </is>
       </c>
     </row>
-    <row r="7" outlineLevel="1" ht="84" customHeight="1">
+    <row r="7" outlineLevel="1" ht="132" customHeight="1">
       <c r="A7" s="10" t="n"/>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>▶ 主输出：物理+混沌双投射物，分裂+无限连锁受诅咒目标</t>
+          <t>★ 造成(9—279)至(14—418)物理傷害
+★ 投射物數量詞綴套用至投射物裂化目標數量
+★ 投射物會朝2個目標分裂
+★ 可從任意數量的受詛咒目標連鎖
+★ 增加50%連鎖範圍
+★ 造成(8—244)至(15—453)混沌傷害
+★ base is projectile 1
+★ can perform skill while moving 1
+▶ 主输出：物理+混沌双投射物，分裂+无限连锁受诅咒目标</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>▶ 寂缠弹：施法速度换更多伤害</t>
+          <t>★ 被輔助法術技能的施放速度減少15%
+★ 被輔助的法術造成35%更多傷害
+▶ 寂缠弹：施法速度换更多伤害</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
@@ -2008,8 +2045,7 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>生命痕跡
-(Level)
+          <t>Life Remnants
 Lv.20</t>
         </is>
       </c>
@@ -2030,18 +2066,11 @@
         </is>
       </c>
     </row>
-    <row r="12" outlineLevel="1" ht="124" customHeight="1">
+    <row r="12" outlineLevel="1" ht="84" customHeight="1">
       <c r="A12" s="10" t="n"/>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>★ 痕跡持續8秒
-★ 擊殺一名敵人時有25%機率生成一個痕跡
-★ 擊中敵人時產生1個痕跡，每3秒只能產生一個
-★ 每個痕跡賦予(11—410)生命
-★ base deal no damage 1
-★ base deal no damage over time 1
-★ skill desired amount override 1
-▶ 血法师赋予：生命痕跡回复</t>
+          <t>▶ 血法师赋予：生命痕跡回复</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
@@ -2162,8 +2191,7 @@
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>衰弱
-(Level)</t>
+          <t>Enfeeble</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
@@ -2227,18 +2255,7 @@
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>■ 將你的衰弱替換成腥紅特效。
-■ 賦予技能: 招架
-■ 輕盾: 格擋時，會對敵人施加衰弱衰弱詛咒
-★ 1.5秒延遲後施加詛咒
-★ 詛咒無法套用至等級高於(0—20)的敵人
-★ 詛咒範圍為(1.5—3.1)公尺
-★ 詛咒使目標造成(20—29)%更少傷害
-★ 詛咒持續時間為(6—7.4)秒
-★ base deal no damage 1
-★ can perform skill while moving 1
-★ movement speed +% final while performing action -70
-▶ Blasphemy 减伤诅咒</t>
+          <t>▶ Blasphemy 减伤诅咒</t>
         </is>
       </c>
       <c r="F18" s="11" t="inlineStr">
@@ -2261,8 +2278,7 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>凋零光環
-(Level)
+          <t>Withering Presence
 Lv.18</t>
         </is>
       </c>
@@ -2278,14 +2294,11 @@
         </is>
       </c>
     </row>
-    <row r="21" outlineLevel="1" ht="92" customHeight="1">
+    <row r="21" outlineLevel="1" ht="76" customHeight="1">
       <c r="A21" s="10" t="n"/>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>★ 凋零持續時間為6秒
-★ 身處你存在範圍中的敵人每(1.42—1.8)秒承受凋零
-★ skill desired amount override 1
-▶ 凋零 debuff 叠层</t>
+          <t>▶ 凋零 debuff 叠层</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
@@ -2499,8 +2512,7 @@
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>狙擊者印記
-(Level)
+          <t>Sniper's Mark
 Lv.18</t>
         </is>
       </c>
@@ -2520,19 +2532,11 @@
         </is>
       </c>
     </row>
-    <row r="32" outlineLevel="1" ht="132" customHeight="1">
+    <row r="32" outlineLevel="1" ht="36" customHeight="1">
       <c r="A32" s="10" t="n"/>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>★ 限制1個標記的目標
-★ 印記持續時間上限為8秒
-★ 下一個對帶有印記敵人的暴擊增加(20—77)%暴擊傷害加成
-★ base deal no damage 1
-★ can perform skill while moving 1
-★ movement speed +% final while performing action -70
-★ movement speed acceleration +% per second while performing action 160
-★ movement speed while performing action locked duration % 50
-▶ 印记技能</t>
+          <t>▶ 印记技能</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
@@ -2584,17 +2588,31 @@
       </c>
       <c r="B36" s="12" t="inlineStr">
         <is>
-          <t>Liminal Coil</t>
+          <t>臨界纏繞
+(Liminal Coil)</t>
         </is>
       </c>
       <c r="C36" s="13" t="n"/>
     </row>
-    <row r="37" outlineLevel="1" ht="72" customHeight="1">
+    <row r="37" outlineLevel="1" ht="264" customHeight="1">
       <c r="A37" s="10" t="n"/>
       <c r="B37" s="11" t="inlineStr"/>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Liminal Coil
+          <t>臨界纏繞 (Liminal Coil)
+底材：Twisted Wand
+需求:  等級 65, 114 智慧
+■ 賦予技能: 寂纏彈
+★ 增加(71—113)%法術傷害
+★ 增加(7—13)%施放速度
+★ 你施加的詛咒幅度為零
+★ 你施加的詛咒無視詛咒上限
+★ 目標每受一個詛咒影響，法術擊中即獲得(23—31)%傷害的額外混沌傷害
+★ 目標每受一個詛咒影響，法術擊中即獲得(23—31)%傷害的額外物理傷害
+「In that moment, Viridi's bones became 
+branches, weaving over the Darkness. 
+She coiled around the nothing, 
+trapping it within her everything.」
 ▶ BD 用途：BD 核心：赋予寂缠弹；诅咒幅度归零但无视诅咒上限，每诅咒巨额额外物理/混沌
 🔗 https://poe2db.tw/tw/Liminal_Coil
 ▶ 唯一来源寂缠弹；6 诅咒各 +25~31% 额外物理/混沌</t>
@@ -2610,17 +2628,27 @@
       </c>
       <c r="B39" s="12" t="inlineStr">
         <is>
-          <t>Alpha's Howl</t>
+          <t>極地之嗥
+(Alpha's Howl)</t>
         </is>
       </c>
       <c r="C39" s="13" t="n"/>
     </row>
-    <row r="40" outlineLevel="1" ht="72" customHeight="1">
+    <row r="40" outlineLevel="1" ht="204" customHeight="1">
       <c r="A40" s="10" t="n"/>
       <c r="B40" s="11" t="inlineStr"/>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Alpha's Howl
+          <t>極地之嗥 (Alpha's Howl)
+底材：Armoured Cap
+需求:  等級 65, 91 敏捷
+★ 增加(80—100)%閃避值
+★ +100精魂
+★ +(50—75)%冰冷抗性
+★ 存在範圍的範圍加倍
+「Nature respects the strong
+And paints the snow red
+With the blood of the weak」
 ▶ BD 用途：+100 Spirit，Blasphemy 多诅咒必备
 🔗 https://poe2db.tw/tw/Alphas_Howl
 ▶ +100 Spirit，Blasphemy 必备</t>
@@ -2876,17 +2904,27 @@
       </c>
       <c r="B71" s="12" t="inlineStr">
         <is>
-          <t>Effigy of Cruelty</t>
+          <t>殘酷塑像
+(Effigy of Cruelty)</t>
         </is>
       </c>
       <c r="C71" s="13" t="n"/>
     </row>
-    <row r="72" outlineLevel="1" ht="72" customHeight="1">
+    <row r="72" outlineLevel="1" ht="204" customHeight="1">
       <c r="A72" s="10" t="n"/>
       <c r="B72" s="11" t="inlineStr"/>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>Effigy of Cruelty
+          <t>殘酷塑像 (Effigy of Cruelty)
+底材：Antler Focus
+需求:  等級 10, 17 智慧
+★ +(20—30)最大能量護盾
+★ 增加(40—50)%法術傷害
+★ +10點智慧
+★ +(7—13)%混沌抗性
+★ 以法術暴擊時，施加(1—3)層的暴擊弱點
+「The horrors we imagined as children
+still exist somewhere in the dark...」
 ▶ BD 用途：II 组副手：法术暴击叠 Critical Weakness
 🔗 https://poe2db.tw/tw/Effigy_of_Cruelty
 ▶ Entangle 叠 Critical Weakness（冷/混沌变体可选 The Wicked Quill）</t>

</xml_diff>

<commit_message>
Sync BD docs 2026-07-08-v1 (202607160258) from my-cloud-project@b2f77ba
</commit_message>
<xml_diff>
--- a/Coiling_Bolts_Blood_Mage_BD指南.xlsx
+++ b/Coiling_Bolts_Blood_Mage_BD指南.xlsx
@@ -379,7 +379,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>1</col>
       <colOff>0</colOff>
       <row>11</row>
       <rowOff>0</rowOff>
@@ -404,9 +404,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>4</col>
       <colOff>0</colOff>
-      <row>14</row>
+      <row>11</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -431,7 +431,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>17</row>
+      <row>14</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -454,7 +454,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>2</col>
+      <col>1</col>
       <colOff>0</colOff>
       <row>17</row>
       <rowOff>0</rowOff>
@@ -479,7 +479,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>3</col>
+      <col>2</col>
       <colOff>0</colOff>
       <row>17</row>
       <rowOff>0</rowOff>
@@ -504,9 +504,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>2</col>
+      <col>3</col>
       <colOff>0</colOff>
-      <row>20</row>
+      <row>17</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -529,9 +529,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>4</col>
       <colOff>0</colOff>
-      <row>25</row>
+      <row>17</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -556,7 +556,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>28</row>
+      <row>20</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -579,12 +579,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>2</col>
       <colOff>0</colOff>
-      <row>36</row>
+      <row>20</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="200025" cy="609600"/>
+    <ext cx="609600" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="13" name="Image 13" descr="Picture"/>
@@ -606,7 +606,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>39</row>
+      <row>25</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -631,7 +631,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>71</row>
+      <row>28</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -642,6 +642,106 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId15"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>31</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="16" name="Image 16" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId16"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>36</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="200025" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId17"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>39</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="18" name="Image 18" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId18"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>71</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="19" name="Image 19" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId19"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2045,7 +2145,8 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Life Remnants
+          <t>生命痕跡
+(Level)
 Lv.20</t>
         </is>
       </c>
@@ -2066,11 +2167,18 @@
         </is>
       </c>
     </row>
-    <row r="12" outlineLevel="1" ht="84" customHeight="1">
+    <row r="12" outlineLevel="1" ht="124" customHeight="1">
       <c r="A12" s="10" t="n"/>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>▶ 血法师赋予：生命痕跡回复</t>
+          <t>★ 痕跡持續8秒
+★ 擊殺一名敵人時有25%機率生成一個痕跡
+★ 擊中敵人時產生1個痕跡，每3秒只能產生一個
+★ 每個痕跡賦予(11—410)生命
+★ base deal no damage 1
+★ base deal no damage over time 1
+★ skill desired amount override 1
+▶ 血法师赋予：生命痕跡回复</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
@@ -2191,7 +2299,8 @@
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>Enfeeble</t>
+          <t>衰弱
+(Level)</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
@@ -2255,7 +2364,18 @@
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>▶ Blasphemy 减伤诅咒</t>
+          <t>■ 將你的衰弱替換成腥紅特效。
+■ 賦予技能: 招架
+■ 輕盾: 格擋時，會對敵人施加衰弱衰弱詛咒
+★ 1.5秒延遲後施加詛咒
+★ 詛咒無法套用至等級高於(0—20)的敵人
+★ 詛咒範圍為(1.5—3.1)公尺
+★ 詛咒使目標造成(20—29)%更少傷害
+★ 詛咒持續時間為(6—7.4)秒
+★ base deal no damage 1
+★ can perform skill while moving 1
+★ movement speed +% final while performing action -70
+▶ Blasphemy 减伤诅咒</t>
         </is>
       </c>
       <c r="F18" s="11" t="inlineStr">
@@ -2278,7 +2398,8 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Withering Presence
+          <t>凋零光環
+(Level)
 Lv.18</t>
         </is>
       </c>
@@ -2294,11 +2415,14 @@
         </is>
       </c>
     </row>
-    <row r="21" outlineLevel="1" ht="76" customHeight="1">
+    <row r="21" outlineLevel="1" ht="92" customHeight="1">
       <c r="A21" s="10" t="n"/>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>▶ 凋零 debuff 叠层</t>
+          <t>★ 凋零持續時間為6秒
+★ 身處你存在範圍中的敵人每(1.42—1.8)秒承受凋零
+★ skill desired amount override 1
+▶ 凋零 debuff 叠层</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
@@ -2512,7 +2636,8 @@
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>Sniper's Mark
+          <t>狙擊者印記
+(Level)
 Lv.18</t>
         </is>
       </c>
@@ -2532,11 +2657,19 @@
         </is>
       </c>
     </row>
-    <row r="32" outlineLevel="1" ht="36" customHeight="1">
+    <row r="32" outlineLevel="1" ht="132" customHeight="1">
       <c r="A32" s="10" t="n"/>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>▶ 印记技能</t>
+          <t>★ 限制1個標記的目標
+★ 印記持續時間上限為8秒
+★ 下一個對帶有印記敵人的暴擊增加(20—77)%暴擊傷害加成
+★ base deal no damage 1
+★ can perform skill while moving 1
+★ movement speed +% final while performing action -70
+★ movement speed acceleration +% per second while performing action 160
+★ movement speed while performing action locked duration % 50
+▶ 印记技能</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Sync BD docs 2026-07-08-v1 (202607160305) from my-cloud-project@11798af
</commit_message>
<xml_diff>
--- a/Coiling_Bolts_Blood_Mage_BD指南.xlsx
+++ b/Coiling_Bolts_Blood_Mage_BD指南.xlsx
@@ -279,7 +279,7 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>3</col>
       <colOff>0</colOff>
       <row>6</row>
       <rowOff>0</rowOff>
@@ -304,7 +304,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>2</col>
+      <col>4</col>
       <colOff>0</colOff>
       <row>6</row>
       <rowOff>0</rowOff>
@@ -329,9 +329,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>3</col>
+      <col>4</col>
       <colOff>0</colOff>
-      <row>6</row>
+      <row>11</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -354,9 +354,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>2</col>
       <colOff>0</colOff>
-      <row>6</row>
+      <row>20</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -367,381 +367,6 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId4"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>11</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="5" name="Image 5" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId5"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>0</colOff>
-      <row>11</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="6" name="Image 6" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId6"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>14</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="7" name="Image 7" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId7"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>17</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="8" name="Image 8" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId8"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>17</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="9" name="Image 9" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId9"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>3</col>
-      <colOff>0</colOff>
-      <row>17</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="10" name="Image 10" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId10"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>0</colOff>
-      <row>17</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="11" name="Image 11" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId11"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>20</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="12" name="Image 12" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId12"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>20</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="13" name="Image 13" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId13"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>25</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="14" name="Image 14" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId14"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>28</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="15" name="Image 15" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId15"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>31</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="16" name="Image 16" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId16"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>36</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="200025" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="17" name="Image 17" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId17"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>39</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="18" name="Image 18" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId18"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>71</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="19" name="Image 19" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId19"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2031,15 +1656,13 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>寂纏彈
-(Level)
+          <t>Coiling Bolts
 Lv.20</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>細思施法
-(Considered Casting)</t>
+          <t>Considered Casting</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
@@ -2065,26 +1688,16 @@
         </is>
       </c>
     </row>
-    <row r="7" outlineLevel="1" ht="132" customHeight="1">
+    <row r="7" outlineLevel="1" ht="84" customHeight="1">
       <c r="A7" s="10" t="n"/>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>★ 造成(9—279)至(14—418)物理傷害
-★ 投射物數量詞綴套用至投射物裂化目標數量
-★ 投射物會朝2個目標分裂
-★ 可從任意數量的受詛咒目標連鎖
-★ 增加50%連鎖範圍
-★ 造成(8—244)至(15—453)混沌傷害
-★ base is projectile 1
-★ can perform skill while moving 1
-▶ 主输出：物理+混沌双投射物，分裂+无限连锁受诅咒目标</t>
+          <t>▶ 主输出：物理+混沌双投射物，分裂+无限连锁受诅咒目标</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>★ 被輔助法術技能的施放速度減少15%
-★ 被輔助的法術造成35%更多傷害
-▶ 寂缠弹：施法速度换更多伤害</t>
+          <t>▶ 寂缠弹：施法速度换更多伤害</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
@@ -2145,8 +1758,7 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>生命痕跡
-(Level)
+          <t>Life Remnants
 Lv.20</t>
         </is>
       </c>
@@ -2167,18 +1779,11 @@
         </is>
       </c>
     </row>
-    <row r="12" outlineLevel="1" ht="124" customHeight="1">
+    <row r="12" outlineLevel="1" ht="84" customHeight="1">
       <c r="A12" s="10" t="n"/>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>★ 痕跡持續8秒
-★ 擊殺一名敵人時有25%機率生成一個痕跡
-★ 擊中敵人時產生1個痕跡，每3秒只能產生一個
-★ 每個痕跡賦予(11—410)生命
-★ base deal no damage 1
-★ base deal no damage over time 1
-★ skill desired amount override 1
-▶ 血法师赋予：生命痕跡回复</t>
+          <t>▶ 血法师赋予：生命痕跡回复</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
@@ -2208,8 +1813,7 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>咒符之力
-(Level)
+          <t>Sigil of Power
 Lv.18</t>
         </is>
       </c>
@@ -2234,20 +1838,11 @@
         </is>
       </c>
     </row>
-    <row r="15" outlineLevel="1" ht="140" customHeight="1">
+    <row r="15" outlineLevel="1" ht="36" customHeight="1">
       <c r="A15" s="10" t="n"/>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>■ 將技能「咒符之力」的特效替換為聖能。
-★ 疊層間至少1秒
-★ 符印範圍為3公尺
-★ 在區域中共消耗50%最大魔力時，獲得1個疊層
-★ 符印持續時間為(10—11.9)秒
-★ 疊層上限4
-★ 每層增益效果賦予(10—14)%更多法術傷害
-★ base number of sigil of power allowed 1
-★ can perform skill while moving 1
-▶ Boss 前铺设增伤法阵</t>
+          <t>▶ Boss 前铺设增伤法阵</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
@@ -2280,27 +1875,23 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>瀆神
-(Level)
+          <t>Blasphemy
 Lv.19</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>時空鎖鏈
-(Level)</t>
+          <t>Temporal Chains</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>元素要害
-(Level)</t>
+          <t>Elemental Weakness</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>衰弱
-(Level)</t>
+          <t>Enfeeble</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
@@ -2314,68 +1905,26 @@
         </is>
       </c>
     </row>
-    <row r="18" outlineLevel="1" ht="164" customHeight="1">
+    <row r="18" outlineLevel="1" ht="36" customHeight="1">
       <c r="A18" s="10" t="n"/>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>■ 移除玩家極地裝甲、暴風之盾、鮮血狂怒、熔岩護盾、迷蹤、石化之血、光環、病疫之難、凋零之步、詛咒和捷光環的視覺特效。
-■ 你的光環特效替換為力場防護罩。
-■ 你的光環特效替換為一個閃耀著電光的骷髏。
-■ 你的光環特效替還為一個被地獄之火圍繞的骷髏。
-★ 插槽中的詛咒技能會以光環的形式影響周圍
-★ 每個插槽中的詛咒占用60精魂
-★ 被輔助的詛咒有(41—50)%更少效果幅度
-★ 插槽中的技能在基礎範圍上額外增加+1公尺
-★ base deal no damage 1
-▶ 诅咒光环</t>
+          <t>▶ 诅咒光环</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>■ 將你的時空鎖鏈替換成腥紅特效。
-■ 將技能「時空鎖鏈」的特效替換為瓦爾時空先知。
-★ 1.5秒延遲後施加詛咒
-★ 詛咒無法套用至等級高於(0—20)的敵人
-★ 詛咒範圍為(1.5—3.1)公尺
-★ 詛咒會緩速目標(40—59)%
-★ 詛咒持續時間為(6—7.4)秒
-★ 詛咒使目標身上其他效果減緩25%失效
-★ base deal no damage 1
-★ can perform skill while moving 1
-▶ Blasphemy 光环诅咒之一</t>
+          <t>▶ Blasphemy 光环诅咒之一</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>■ 將技能「元素要害」的特效替換為深淵。
-■ 將技能「元素要害」的特效替換為幽暗碎魂。
-■ +8%的護甲值也會套用至元素傷害
-■ 能量護盾開始充能速度加快10%
-★ 1.5秒延遲後施加詛咒
-★ 詛咒無法套用至等級高於(0—20)的敵人
-★ 詛咒範圍為(1.5—3.1)公尺
-★ 詛咒使元素抗性(-59—-40)%
-★ 詛咒持續時間為(6—7.4)秒
-★ base deal no damage 1
-★ can perform skill while moving 1
-★ movement speed +% final while performing action -70
-▶ Blasphemy 降抗诅咒</t>
+          <t>▶ Blasphemy 降抗诅咒</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>■ 將你的衰弱替換成腥紅特效。
-■ 賦予技能: 招架
-■ 輕盾: 格擋時，會對敵人施加衰弱衰弱詛咒
-★ 1.5秒延遲後施加詛咒
-★ 詛咒無法套用至等級高於(0—20)的敵人
-★ 詛咒範圍為(1.5—3.1)公尺
-★ 詛咒使目標造成(20—29)%更少傷害
-★ 詛咒持續時間為(6—7.4)秒
-★ base deal no damage 1
-★ can perform skill while moving 1
-★ movement speed +% final while performing action -70
-▶ Blasphemy 减伤诅咒</t>
+          <t>▶ Blasphemy 减伤诅咒</t>
         </is>
       </c>
       <c r="F18" s="11" t="inlineStr">
@@ -2398,8 +1947,7 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>凋零光環
-(Level)
+          <t>Withering Presence
 Lv.18</t>
         </is>
       </c>
@@ -2415,14 +1963,11 @@
         </is>
       </c>
     </row>
-    <row r="21" outlineLevel="1" ht="92" customHeight="1">
+    <row r="21" outlineLevel="1" ht="76" customHeight="1">
       <c r="A21" s="10" t="n"/>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>★ 凋零持續時間為6秒
-★ 身處你存在範圍中的敵人每(1.42—1.8)秒承受凋零
-★ skill desired amount override 1
-▶ 凋零 debuff 叠层</t>
+          <t>▶ 凋零 debuff 叠层</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
@@ -2471,8 +2016,7 @@
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>脆弱
-(Level)
+          <t>Vulnerability
 Lv.19</t>
         </is>
       </c>
@@ -2502,20 +2046,11 @@
         </is>
       </c>
     </row>
-    <row r="26" outlineLevel="1" ht="140" customHeight="1">
+    <row r="26" outlineLevel="1" ht="36" customHeight="1">
       <c r="A26" s="10" t="n"/>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>■ 將你的脆弱替換成腥紅特效。
-★ 1.5秒延遲後施加詛咒
-★ 詛咒無法套用至等級高於(0—20)的敵人
-★ 詛咒範圍為(1.5—3.1)公尺
-★ 詛咒會減少(16—19210)總護甲
-★ 詛咒持續時間為(6—7.4)秒
-★ base deal no damage 1
-★ can perform skill while moving 1
-★ movement speed +% final while performing action -70
-▶ II 组手动诅咒（计入 Liminal 增伤）</t>
+          <t>▶ II 组手动诅咒（计入 Liminal 增伤）</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
@@ -2553,8 +2088,7 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>絕望
-(Level)
+          <t>Despair
 Lv.19</t>
         </is>
       </c>
@@ -2584,21 +2118,11 @@
         </is>
       </c>
     </row>
-    <row r="29" outlineLevel="1" ht="148" customHeight="1">
+    <row r="29" outlineLevel="1" ht="36" customHeight="1">
       <c r="A29" s="10" t="n"/>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>■ 將你的絕望替換成腥紅特效。
-■ 將你的絕望替換成譫妄特效。
-★ 1.5秒延遲後施加詛咒
-★ 詛咒無法套用至等級高於(0—20)的敵人
-★ 詛咒使混沌抗性(-49—-35)%
-★ 詛咒範圍為(1.5—3.1)公尺
-★ 詛咒持續時間為(6—7.4)秒
-★ base deal no damage 1
-★ can perform skill while moving 1
-★ movement speed +% final while performing action -70
-▶ II 组混沌诅咒</t>
+          <t>▶ II 组混沌诅咒</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
@@ -2636,8 +2160,7 @@
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>狙擊者印記
-(Level)
+          <t>Sniper's Mark
 Lv.18</t>
         </is>
       </c>
@@ -2657,19 +2180,11 @@
         </is>
       </c>
     </row>
-    <row r="32" outlineLevel="1" ht="132" customHeight="1">
+    <row r="32" outlineLevel="1" ht="36" customHeight="1">
       <c r="A32" s="10" t="n"/>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>★ 限制1個標記的目標
-★ 印記持續時間上限為8秒
-★ 下一個對帶有印記敵人的暴擊增加(20—77)%暴擊傷害加成
-★ base deal no damage 1
-★ can perform skill while moving 1
-★ movement speed +% final while performing action -70
-★ movement speed acceleration +% per second while performing action 160
-★ movement speed while performing action locked duration % 50
-▶ 印记技能</t>
+          <t>▶ 印记技能</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
@@ -2721,31 +2236,17 @@
       </c>
       <c r="B36" s="12" t="inlineStr">
         <is>
-          <t>臨界纏繞
-(Liminal Coil)</t>
+          <t>Liminal Coil</t>
         </is>
       </c>
       <c r="C36" s="13" t="n"/>
     </row>
-    <row r="37" outlineLevel="1" ht="264" customHeight="1">
+    <row r="37" outlineLevel="1" ht="72" customHeight="1">
       <c r="A37" s="10" t="n"/>
       <c r="B37" s="11" t="inlineStr"/>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>臨界纏繞 (Liminal Coil)
-底材：Twisted Wand
-需求:  等級 65, 114 智慧
-■ 賦予技能: 寂纏彈
-★ 增加(71—113)%法術傷害
-★ 增加(7—13)%施放速度
-★ 你施加的詛咒幅度為零
-★ 你施加的詛咒無視詛咒上限
-★ 目標每受一個詛咒影響，法術擊中即獲得(23—31)%傷害的額外混沌傷害
-★ 目標每受一個詛咒影響，法術擊中即獲得(23—31)%傷害的額外物理傷害
-「In that moment, Viridi's bones became 
-branches, weaving over the Darkness. 
-She coiled around the nothing, 
-trapping it within her everything.」
+          <t>Liminal Coil
 ▶ BD 用途：BD 核心：赋予寂缠弹；诅咒幅度归零但无视诅咒上限，每诅咒巨额额外物理/混沌
 🔗 https://poe2db.tw/tw/Liminal_Coil
 ▶ 唯一来源寂缠弹；6 诅咒各 +25~31% 额外物理/混沌</t>
@@ -2761,27 +2262,17 @@
       </c>
       <c r="B39" s="12" t="inlineStr">
         <is>
-          <t>極地之嗥
-(Alpha's Howl)</t>
+          <t>Alpha's Howl</t>
         </is>
       </c>
       <c r="C39" s="13" t="n"/>
     </row>
-    <row r="40" outlineLevel="1" ht="204" customHeight="1">
+    <row r="40" outlineLevel="1" ht="72" customHeight="1">
       <c r="A40" s="10" t="n"/>
       <c r="B40" s="11" t="inlineStr"/>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>極地之嗥 (Alpha's Howl)
-底材：Armoured Cap
-需求:  等級 65, 91 敏捷
-★ 增加(80—100)%閃避值
-★ +100精魂
-★ +(50—75)%冰冷抗性
-★ 存在範圍的範圍加倍
-「Nature respects the strong
-And paints the snow red
-With the blood of the weak」
+          <t>Alpha's Howl
 ▶ BD 用途：+100 Spirit，Blasphemy 多诅咒必备
 🔗 https://poe2db.tw/tw/Alphas_Howl
 ▶ +100 Spirit，Blasphemy 必备</t>
@@ -3037,27 +2528,17 @@
       </c>
       <c r="B71" s="12" t="inlineStr">
         <is>
-          <t>殘酷塑像
-(Effigy of Cruelty)</t>
+          <t>Effigy of Cruelty</t>
         </is>
       </c>
       <c r="C71" s="13" t="n"/>
     </row>
-    <row r="72" outlineLevel="1" ht="204" customHeight="1">
+    <row r="72" outlineLevel="1" ht="72" customHeight="1">
       <c r="A72" s="10" t="n"/>
       <c r="B72" s="11" t="inlineStr"/>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>殘酷塑像 (Effigy of Cruelty)
-底材：Antler Focus
-需求:  等級 10, 17 智慧
-★ +(20—30)最大能量護盾
-★ 增加(40—50)%法術傷害
-★ +10點智慧
-★ +(7—13)%混沌抗性
-★ 以法術暴擊時，施加(1—3)層的暴擊弱點
-「The horrors we imagined as children
-still exist somewhere in the dark...」
+          <t>Effigy of Cruelty
 ▶ BD 用途：II 组副手：法术暴击叠 Critical Weakness
 🔗 https://poe2db.tw/tw/Effigy_of_Cruelty
 ▶ Entangle 叠 Critical Weakness（冷/混沌变体可选 The Wicked Quill）</t>

</xml_diff>

<commit_message>
Sync BD docs 2026-07-08-v1 (202607160420) from my-cloud-project@97e942d
</commit_message>
<xml_diff>
--- a/Coiling_Bolts_Blood_Mage_BD指南.xlsx
+++ b/Coiling_Bolts_Blood_Mage_BD指南.xlsx
@@ -279,7 +279,7 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>3</col>
+      <col>1</col>
       <colOff>0</colOff>
       <row>6</row>
       <rowOff>0</rowOff>
@@ -304,7 +304,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>2</col>
       <colOff>0</colOff>
       <row>6</row>
       <rowOff>0</rowOff>
@@ -329,9 +329,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>3</col>
       <colOff>0</colOff>
-      <row>11</row>
+      <row>6</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -354,9 +354,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>2</col>
+      <col>4</col>
       <colOff>0</colOff>
-      <row>20</row>
+      <row>6</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -367,6 +367,381 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="10" name="Image 10" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="11" name="Image 11" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="13" name="Image 13" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="14" name="Image 14" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId14"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>28</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId15"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>31</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="16" name="Image 16" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId16"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>36</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="200025" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId17"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>39</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="18" name="Image 18" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId18"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>71</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="19" name="Image 19" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId19"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1656,13 +2031,15 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Coiling Bolts
+          <t>寂纏彈
+(Level)
 Lv.20</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Considered Casting</t>
+          <t>細思施法
+(Considered Casting)</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
@@ -1688,16 +2065,26 @@
         </is>
       </c>
     </row>
-    <row r="7" outlineLevel="1" ht="84" customHeight="1">
+    <row r="7" outlineLevel="1" ht="132" customHeight="1">
       <c r="A7" s="10" t="n"/>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>▶ 主输出：物理+混沌双投射物，分裂+无限连锁受诅咒目标</t>
+          <t>★ 造成(9—279)至(14—418)物理傷害
+★ 投射物數量詞綴套用至投射物裂化目標數量
+★ 投射物會朝2個目標分裂
+★ 可從任意數量的受詛咒目標連鎖
+★ 增加50%連鎖範圍
+★ 造成(8—244)至(15—453)混沌傷害
+★ base is projectile 1
+★ can perform skill while moving 1
+▶ 主输出：物理+混沌双投射物，分裂+无限连锁受诅咒目标</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>▶ 寂缠弹：施法速度换更多伤害</t>
+          <t>★ 被輔助法術技能的施放速度減少15%
+★ 被輔助的法術造成35%更多傷害
+▶ 寂缠弹：施法速度换更多伤害</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
@@ -1758,7 +2145,8 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Life Remnants
+          <t>生命痕跡
+(Level)
 Lv.20</t>
         </is>
       </c>
@@ -1779,11 +2167,18 @@
         </is>
       </c>
     </row>
-    <row r="12" outlineLevel="1" ht="84" customHeight="1">
+    <row r="12" outlineLevel="1" ht="124" customHeight="1">
       <c r="A12" s="10" t="n"/>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>▶ 血法师赋予：生命痕跡回复</t>
+          <t>★ 痕跡持續8秒
+★ 擊殺一名敵人時有25%機率生成一個痕跡
+★ 擊中敵人時產生1個痕跡，每3秒只能產生一個
+★ 每個痕跡賦予(11—410)生命
+★ base deal no damage 1
+★ base deal no damage over time 1
+★ skill desired amount override 1
+▶ 血法师赋予：生命痕跡回复</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
@@ -1813,7 +2208,8 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>Sigil of Power
+          <t>咒符之力
+(Level)
 Lv.18</t>
         </is>
       </c>
@@ -1838,11 +2234,20 @@
         </is>
       </c>
     </row>
-    <row r="15" outlineLevel="1" ht="36" customHeight="1">
+    <row r="15" outlineLevel="1" ht="140" customHeight="1">
       <c r="A15" s="10" t="n"/>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>▶ Boss 前铺设增伤法阵</t>
+          <t>■ 將技能「咒符之力」的特效替換為聖能。
+★ 疊層間至少1秒
+★ 符印範圍為3公尺
+★ 在區域中共消耗50%最大魔力時，獲得1個疊層
+★ 符印持續時間為(10—11.9)秒
+★ 疊層上限4
+★ 每層增益效果賦予(10—14)%更多法術傷害
+★ base number of sigil of power allowed 1
+★ can perform skill while moving 1
+▶ Boss 前铺设增伤法阵</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
@@ -1875,23 +2280,27 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>Blasphemy
+          <t>瀆神
+(Level)
 Lv.19</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>Temporal Chains</t>
+          <t>時空鎖鏈
+(Level)</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>Elemental Weakness</t>
+          <t>元素要害
+(Level)</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>Enfeeble</t>
+          <t>衰弱
+(Level)</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
@@ -1905,26 +2314,68 @@
         </is>
       </c>
     </row>
-    <row r="18" outlineLevel="1" ht="36" customHeight="1">
+    <row r="18" outlineLevel="1" ht="164" customHeight="1">
       <c r="A18" s="10" t="n"/>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>▶ 诅咒光环</t>
+          <t>■ 移除玩家極地裝甲、暴風之盾、鮮血狂怒、熔岩護盾、迷蹤、石化之血、光環、病疫之難、凋零之步、詛咒和捷光環的視覺特效。
+■ 你的光環特效替換為力場防護罩。
+■ 你的光環特效替換為一個閃耀著電光的骷髏。
+■ 你的光環特效替還為一個被地獄之火圍繞的骷髏。
+★ 插槽中的詛咒技能會以光環的形式影響周圍
+★ 每個插槽中的詛咒占用60精魂
+★ 被輔助的詛咒有(41—50)%更少效果幅度
+★ 插槽中的技能在基礎範圍上額外增加+1公尺
+★ base deal no damage 1
+▶ 诅咒光环</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>▶ Blasphemy 光环诅咒之一</t>
+          <t>■ 將你的時空鎖鏈替換成腥紅特效。
+■ 將技能「時空鎖鏈」的特效替換為瓦爾時空先知。
+★ 1.5秒延遲後施加詛咒
+★ 詛咒無法套用至等級高於(0—20)的敵人
+★ 詛咒範圍為(1.5—3.1)公尺
+★ 詛咒會緩速目標(40—59)%
+★ 詛咒持續時間為(6—7.4)秒
+★ 詛咒使目標身上其他效果減緩25%失效
+★ base deal no damage 1
+★ can perform skill while moving 1
+▶ Blasphemy 光环诅咒之一</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>▶ Blasphemy 降抗诅咒</t>
+          <t>■ 將技能「元素要害」的特效替換為深淵。
+■ 將技能「元素要害」的特效替換為幽暗碎魂。
+■ +8%的護甲值也會套用至元素傷害
+■ 能量護盾開始充能速度加快10%
+★ 1.5秒延遲後施加詛咒
+★ 詛咒無法套用至等級高於(0—20)的敵人
+★ 詛咒範圍為(1.5—3.1)公尺
+★ 詛咒使元素抗性(-59—-40)%
+★ 詛咒持續時間為(6—7.4)秒
+★ base deal no damage 1
+★ can perform skill while moving 1
+★ movement speed +% final while performing action -70
+▶ Blasphemy 降抗诅咒</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>▶ Blasphemy 减伤诅咒</t>
+          <t>■ 將你的衰弱替換成腥紅特效。
+■ 賦予技能: 招架
+■ 輕盾: 格擋時，會對敵人施加衰弱衰弱詛咒
+★ 1.5秒延遲後施加詛咒
+★ 詛咒無法套用至等級高於(0—20)的敵人
+★ 詛咒範圍為(1.5—3.1)公尺
+★ 詛咒使目標造成(20—29)%更少傷害
+★ 詛咒持續時間為(6—7.4)秒
+★ base deal no damage 1
+★ can perform skill while moving 1
+★ movement speed +% final while performing action -70
+▶ Blasphemy 减伤诅咒</t>
         </is>
       </c>
       <c r="F18" s="11" t="inlineStr">
@@ -1947,7 +2398,8 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Withering Presence
+          <t>凋零光環
+(Level)
 Lv.18</t>
         </is>
       </c>
@@ -1963,11 +2415,14 @@
         </is>
       </c>
     </row>
-    <row r="21" outlineLevel="1" ht="76" customHeight="1">
+    <row r="21" outlineLevel="1" ht="92" customHeight="1">
       <c r="A21" s="10" t="n"/>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>▶ 凋零 debuff 叠层</t>
+          <t>★ 凋零持續時間為6秒
+★ 身處你存在範圍中的敵人每(1.42—1.8)秒承受凋零
+★ skill desired amount override 1
+▶ 凋零 debuff 叠层</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
@@ -2016,7 +2471,8 @@
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>Vulnerability
+          <t>脆弱
+(Level)
 Lv.19</t>
         </is>
       </c>
@@ -2046,11 +2502,20 @@
         </is>
       </c>
     </row>
-    <row r="26" outlineLevel="1" ht="36" customHeight="1">
+    <row r="26" outlineLevel="1" ht="140" customHeight="1">
       <c r="A26" s="10" t="n"/>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>▶ II 组手动诅咒（计入 Liminal 增伤）</t>
+          <t>■ 將你的脆弱替換成腥紅特效。
+★ 1.5秒延遲後施加詛咒
+★ 詛咒無法套用至等級高於(0—20)的敵人
+★ 詛咒範圍為(1.5—3.1)公尺
+★ 詛咒會減少(16—19210)總護甲
+★ 詛咒持續時間為(6—7.4)秒
+★ base deal no damage 1
+★ can perform skill while moving 1
+★ movement speed +% final while performing action -70
+▶ II 组手动诅咒（计入 Liminal 增伤）</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
@@ -2088,7 +2553,8 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Despair
+          <t>絕望
+(Level)
 Lv.19</t>
         </is>
       </c>
@@ -2118,11 +2584,21 @@
         </is>
       </c>
     </row>
-    <row r="29" outlineLevel="1" ht="36" customHeight="1">
+    <row r="29" outlineLevel="1" ht="148" customHeight="1">
       <c r="A29" s="10" t="n"/>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>▶ II 组混沌诅咒</t>
+          <t>■ 將你的絕望替換成腥紅特效。
+■ 將你的絕望替換成譫妄特效。
+★ 1.5秒延遲後施加詛咒
+★ 詛咒無法套用至等級高於(0—20)的敵人
+★ 詛咒使混沌抗性(-49—-35)%
+★ 詛咒範圍為(1.5—3.1)公尺
+★ 詛咒持續時間為(6—7.4)秒
+★ base deal no damage 1
+★ can perform skill while moving 1
+★ movement speed +% final while performing action -70
+▶ II 组混沌诅咒</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
@@ -2160,7 +2636,8 @@
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>Sniper's Mark
+          <t>狙擊者印記
+(Level)
 Lv.18</t>
         </is>
       </c>
@@ -2180,11 +2657,19 @@
         </is>
       </c>
     </row>
-    <row r="32" outlineLevel="1" ht="36" customHeight="1">
+    <row r="32" outlineLevel="1" ht="132" customHeight="1">
       <c r="A32" s="10" t="n"/>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>▶ 印记技能</t>
+          <t>★ 限制1個標記的目標
+★ 印記持續時間上限為8秒
+★ 下一個對帶有印記敵人的暴擊增加(20—77)%暴擊傷害加成
+★ base deal no damage 1
+★ can perform skill while moving 1
+★ movement speed +% final while performing action -70
+★ movement speed acceleration +% per second while performing action 160
+★ movement speed while performing action locked duration % 50
+▶ 印记技能</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
@@ -2236,17 +2721,31 @@
       </c>
       <c r="B36" s="12" t="inlineStr">
         <is>
-          <t>Liminal Coil</t>
+          <t>臨界纏繞
+(Liminal Coil)</t>
         </is>
       </c>
       <c r="C36" s="13" t="n"/>
     </row>
-    <row r="37" outlineLevel="1" ht="72" customHeight="1">
+    <row r="37" outlineLevel="1" ht="264" customHeight="1">
       <c r="A37" s="10" t="n"/>
       <c r="B37" s="11" t="inlineStr"/>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Liminal Coil
+          <t>臨界纏繞 (Liminal Coil)
+底材：Twisted Wand
+需求:  等級 65, 114 智慧
+■ 賦予技能: 寂纏彈
+★ 增加(71—113)%法術傷害
+★ 增加(7—13)%施放速度
+★ 你施加的詛咒幅度為零
+★ 你施加的詛咒無視詛咒上限
+★ 目標每受一個詛咒影響，法術擊中即獲得(23—31)%傷害的額外混沌傷害
+★ 目標每受一個詛咒影響，法術擊中即獲得(23—31)%傷害的額外物理傷害
+「In that moment, Viridi's bones became 
+branches, weaving over the Darkness. 
+She coiled around the nothing, 
+trapping it within her everything.」
 ▶ BD 用途：BD 核心：赋予寂缠弹；诅咒幅度归零但无视诅咒上限，每诅咒巨额额外物理/混沌
 🔗 https://poe2db.tw/tw/Liminal_Coil
 ▶ 唯一来源寂缠弹；6 诅咒各 +25~31% 额外物理/混沌</t>
@@ -2262,17 +2761,27 @@
       </c>
       <c r="B39" s="12" t="inlineStr">
         <is>
-          <t>Alpha's Howl</t>
+          <t>極地之嗥
+(Alpha's Howl)</t>
         </is>
       </c>
       <c r="C39" s="13" t="n"/>
     </row>
-    <row r="40" outlineLevel="1" ht="72" customHeight="1">
+    <row r="40" outlineLevel="1" ht="204" customHeight="1">
       <c r="A40" s="10" t="n"/>
       <c r="B40" s="11" t="inlineStr"/>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Alpha's Howl
+          <t>極地之嗥 (Alpha's Howl)
+底材：Armoured Cap
+需求:  等級 65, 91 敏捷
+★ 增加(80—100)%閃避值
+★ +100精魂
+★ +(50—75)%冰冷抗性
+★ 存在範圍的範圍加倍
+「Nature respects the strong
+And paints the snow red
+With the blood of the weak」
 ▶ BD 用途：+100 Spirit，Blasphemy 多诅咒必备
 🔗 https://poe2db.tw/tw/Alphas_Howl
 ▶ +100 Spirit，Blasphemy 必备</t>
@@ -2528,17 +3037,27 @@
       </c>
       <c r="B71" s="12" t="inlineStr">
         <is>
-          <t>Effigy of Cruelty</t>
+          <t>殘酷塑像
+(Effigy of Cruelty)</t>
         </is>
       </c>
       <c r="C71" s="13" t="n"/>
     </row>
-    <row r="72" outlineLevel="1" ht="72" customHeight="1">
+    <row r="72" outlineLevel="1" ht="204" customHeight="1">
       <c r="A72" s="10" t="n"/>
       <c r="B72" s="11" t="inlineStr"/>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>Effigy of Cruelty
+          <t>殘酷塑像 (Effigy of Cruelty)
+底材：Antler Focus
+需求:  等級 10, 17 智慧
+★ +(20—30)最大能量護盾
+★ 增加(40—50)%法術傷害
+★ +10點智慧
+★ +(7—13)%混沌抗性
+★ 以法術暴擊時，施加(1—3)層的暴擊弱點
+「The horrors we imagined as children
+still exist somewhere in the dark...」
 ▶ BD 用途：II 组副手：法术暴击叠 Critical Weakness
 🔗 https://poe2db.tw/tw/Effigy_of_Cruelty
 ▶ Entangle 叠 Critical Weakness（冷/混沌变体可选 The Wicked Quill）</t>

</xml_diff>

<commit_message>
Sync BD docs 2026-07-08-v1 (202607160950) from my-cloud-project@2d7e3e5
</commit_message>
<xml_diff>
--- a/Coiling_Bolts_Blood_Mage_BD指南.xlsx
+++ b/Coiling_Bolts_Blood_Mage_BD指南.xlsx
@@ -454,7 +454,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>2</col>
       <colOff>0</colOff>
       <row>17</row>
       <rowOff>0</rowOff>
@@ -479,7 +479,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>2</col>
+      <col>3</col>
       <colOff>0</colOff>
       <row>17</row>
       <rowOff>0</rowOff>
@@ -504,7 +504,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>3</col>
+      <col>4</col>
       <colOff>0</colOff>
       <row>17</row>
       <rowOff>0</rowOff>
@@ -529,9 +529,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>1</col>
       <colOff>0</colOff>
-      <row>17</row>
+      <row>20</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -554,7 +554,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>2</col>
       <colOff>0</colOff>
       <row>20</row>
       <rowOff>0</rowOff>
@@ -579,9 +579,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>2</col>
+      <col>1</col>
       <colOff>0</colOff>
-      <row>20</row>
+      <row>25</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -606,7 +606,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>25</row>
+      <row>28</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -631,7 +631,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>28</row>
+      <row>31</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -656,10 +656,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>31</row>
+      <row>36</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="609600" cy="609600"/>
+    <ext cx="200025" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="16" name="Image 16" descr="Picture"/>
@@ -681,10 +681,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>36</row>
+      <row>39</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="200025" cy="609600"/>
+    <ext cx="609600" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="17" name="Image 17" descr="Picture"/>
@@ -706,7 +706,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>39</row>
+      <row>71</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -717,31 +717,6 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId18"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>71</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="19" name="Image 19" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId19"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2280,8 +2255,7 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>瀆神
-(Level)
+          <t>Blasphemy
 Lv.19</t>
         </is>
       </c>
@@ -2318,16 +2292,7 @@
       <c r="A18" s="10" t="n"/>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>■ 移除玩家極地裝甲、暴風之盾、鮮血狂怒、熔岩護盾、迷蹤、石化之血、光環、病疫之難、凋零之步、詛咒和捷光環的視覺特效。
-■ 你的光環特效替換為力場防護罩。
-■ 你的光環特效替換為一個閃耀著電光的骷髏。
-■ 你的光環特效替還為一個被地獄之火圍繞的骷髏。
-★ 插槽中的詛咒技能會以光環的形式影響周圍
-★ 每個插槽中的詛咒占用60精魂
-★ 被輔助的詛咒有(41—50)%更少效果幅度
-★ 插槽中的技能在基礎範圍上額外增加+1公尺
-★ base deal no damage 1
-▶ 诅咒光环</t>
+          <t>▶ 诅咒光环</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Sync BD docs 2026-07-08-v1 (202607200302) from my-cloud-project@2621394
</commit_message>
<xml_diff>
--- a/Coiling_Bolts_Blood_Mage_BD指南.xlsx
+++ b/Coiling_Bolts_Blood_Mage_BD指南.xlsx
@@ -454,7 +454,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>2</col>
+      <col>1</col>
       <colOff>0</colOff>
       <row>17</row>
       <rowOff>0</rowOff>
@@ -479,7 +479,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>3</col>
+      <col>2</col>
       <colOff>0</colOff>
       <row>17</row>
       <rowOff>0</rowOff>
@@ -504,7 +504,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>3</col>
       <colOff>0</colOff>
       <row>17</row>
       <rowOff>0</rowOff>
@@ -529,9 +529,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>4</col>
       <colOff>0</colOff>
-      <row>20</row>
+      <row>17</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -554,7 +554,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>2</col>
+      <col>1</col>
       <colOff>0</colOff>
       <row>20</row>
       <rowOff>0</rowOff>
@@ -579,9 +579,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>2</col>
       <colOff>0</colOff>
-      <row>25</row>
+      <row>20</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -606,7 +606,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>28</row>
+      <row>25</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -631,7 +631,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>31</row>
+      <row>28</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -656,10 +656,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>36</row>
+      <row>31</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="200025" cy="609600"/>
+    <ext cx="609600" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="16" name="Image 16" descr="Picture"/>
@@ -681,10 +681,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>39</row>
+      <row>36</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="609600" cy="609600"/>
+    <ext cx="200025" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="17" name="Image 17" descr="Picture"/>
@@ -706,7 +706,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>71</row>
+      <row>39</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -717,6 +717,31 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId18"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>71</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="19" name="Image 19" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId19"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2255,7 +2280,8 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>Blasphemy
+          <t>瀆神
+(Level)
 Lv.19</t>
         </is>
       </c>
@@ -2292,7 +2318,16 @@
       <c r="A18" s="10" t="n"/>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>▶ 诅咒光环</t>
+          <t>■ 移除玩家極地裝甲、暴風之盾、鮮血狂怒、熔岩護盾、迷蹤、石化之血、光環、病疫之難、凋零之步、詛咒和捷光環的視覺特效。
+■ 你的光環特效替換為力場防護罩。
+■ 你的光環特效替換為一個閃耀著電光的骷髏。
+■ 你的光環特效替還為一個被地獄之火圍繞的骷髏。
+★ 插槽中的詛咒技能會以光環的形式影響周圍
+★ 每個插槽中的詛咒占用60精魂
+★ 被輔助的詛咒有(41—50)%更少效果幅度
+★ 插槽中的技能在基礎範圍上額外增加+1公尺
+★ base deal no damage 1
+▶ 诅咒光环</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Sync BD docs 2026-07-08-v1 (202607200303) from my-cloud-project@29d158e
</commit_message>
<xml_diff>
--- a/Coiling_Bolts_Blood_Mage_BD指南.xlsx
+++ b/Coiling_Bolts_Blood_Mage_BD指南.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="00-目录" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="01-机制" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="02-武器组" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="03-天赋" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="04-常见问题" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00-目录" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01-机制" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02-武器组" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03-天赋" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04-常见问题" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -276,7 +276,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>1</col>
@@ -291,13 +291,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -316,13 +316,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -341,13 +341,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId3"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -366,13 +366,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId4"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -391,13 +391,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId5"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -416,13 +416,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId6"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -441,13 +441,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId7"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -466,13 +466,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId8"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId8"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -491,13 +491,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId9"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId9"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -516,13 +516,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId10"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId10"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -541,13 +541,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId11"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId11"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -566,13 +566,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId12"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId12"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -591,13 +591,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId13"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId13"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -616,13 +616,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId14"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId14"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -641,13 +641,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId15"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId15"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -666,13 +666,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId16"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId16"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -691,13 +691,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId17"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId17"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -716,13 +716,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId18"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId18"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -741,13 +741,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId19"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId19"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2742,9 +2742,9 @@
 ★ 你施加的詛咒無視詛咒上限
 ★ 目標每受一個詛咒影響，法術擊中即獲得(23—31)%傷害的額外混沌傷害
 ★ 目標每受一個詛咒影響，法術擊中即獲得(23—31)%傷害的額外物理傷害
-「In that moment, Viridi's bones became 
-branches, weaving over the Darkness. 
-She coiled around the nothing, 
+「In that moment, Viridi's bones became 
+branches, weaving over the Darkness. 
+She coiled around the nothing, 
 trapping it within her everything.」
 ▶ BD 用途：BD 核心：赋予寂缠弹；诅咒幅度归零但无视诅咒上限，每诅咒巨额额外物理/混沌
 🔗 https://poe2db.tw/tw/Liminal_Coil
@@ -2779,8 +2779,8 @@
 ★ +100精魂
 ★ +(50—75)%冰冷抗性
 ★ 存在範圍的範圍加倍
-「Nature respects the strong
-And paints the snow red
+「Nature respects the strong
+And paints the snow red
 With the blood of the weak」
 ▶ BD 用途：+100 Spirit，Blasphemy 多诅咒必备
 🔗 https://poe2db.tw/tw/Alphas_Howl
@@ -3056,7 +3056,7 @@
 ★ +10點智慧
 ★ +(7—13)%混沌抗性
 ★ 以法術暴擊時，施加(1—3)層的暴擊弱點
-「The horrors we imagined as children
+「The horrors we imagined as children
 still exist somewhere in the dark...」
 ▶ BD 用途：II 组副手：法术暴击叠 Critical Weakness
 🔗 https://poe2db.tw/tw/Effigy_of_Cruelty

</xml_diff>

<commit_message>
Sync BD docs 2026-07-08-v1 (202607200303) from my-cloud-project@88310eb
</commit_message>
<xml_diff>
--- a/Coiling_Bolts_Blood_Mage_BD指南.xlsx
+++ b/Coiling_Bolts_Blood_Mage_BD指南.xlsx
@@ -404,9 +404,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>1</col>
       <colOff>0</colOff>
-      <row>11</row>
+      <row>17</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -429,9 +429,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>2</col>
       <colOff>0</colOff>
-      <row>14</row>
+      <row>20</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -456,7 +456,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>17</row>
+      <row>31</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -479,12 +479,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>2</col>
+      <col>1</col>
       <colOff>0</colOff>
-      <row>17</row>
+      <row>36</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="609600" cy="609600"/>
+    <ext cx="200025" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="9" name="Image 9" descr="Picture"/>
@@ -504,9 +504,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>3</col>
+      <col>1</col>
       <colOff>0</colOff>
-      <row>17</row>
+      <row>39</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -529,9 +529,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>1</col>
       <colOff>0</colOff>
-      <row>17</row>
+      <row>71</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -542,206 +542,6 @@
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId11"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>20</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="12" name="Image 12" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId12"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>20</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="13" name="Image 13" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId13"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>25</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="14" name="Image 14" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId14"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>28</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="15" name="Image 15" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId15"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>31</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="16" name="Image 16" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId16"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>36</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="200025" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="17" name="Image 17" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId17"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>39</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="18" name="Image 18" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId18"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>71</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="19" name="Image 19" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId19"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2162,8 +1962,7 @@
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>卡塔爾的恢復
-(Date)</t>
+          <t>Khatal's Rejuvenation</t>
         </is>
       </c>
     </row>
@@ -2193,9 +1992,7 @@
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>★ 被輔助技能所創造的痕跡會在拾取時賦予卡塔爾的回春
-★ base_cooldown_speed_+%
-▶ 生命痕跡族裔辅助</t>
+          <t>▶ 生命痕跡族裔辅助</t>
         </is>
       </c>
     </row>
@@ -2208,8 +2005,7 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>咒符之力
-(Level)
+          <t>Sigil of Power
 Lv.18</t>
         </is>
       </c>
@@ -2234,20 +2030,11 @@
         </is>
       </c>
     </row>
-    <row r="15" outlineLevel="1" ht="140" customHeight="1">
+    <row r="15" outlineLevel="1" ht="36" customHeight="1">
       <c r="A15" s="10" t="n"/>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>■ 將技能「咒符之力」的特效替換為聖能。
-★ 疊層間至少1秒
-★ 符印範圍為3公尺
-★ 在區域中共消耗50%最大魔力時，獲得1個疊層
-★ 符印持續時間為(10—11.9)秒
-★ 疊層上限4
-★ 每層增益效果賦予(10—14)%更多法術傷害
-★ base number of sigil of power allowed 1
-★ can perform skill while moving 1
-▶ Boss 前铺设增伤法阵</t>
+          <t>▶ Boss 前铺设增伤法阵</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
@@ -2287,20 +2074,17 @@
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>時空鎖鏈
-(Level)</t>
+          <t>Temporal Chains</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>元素要害
-(Level)</t>
+          <t>Elemental Weakness</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>衰弱
-(Level)</t>
+          <t>Enfeeble</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
@@ -2314,7 +2098,7 @@
         </is>
       </c>
     </row>
-    <row r="18" outlineLevel="1" ht="164" customHeight="1">
+    <row r="18" outlineLevel="1" ht="140" customHeight="1">
       <c r="A18" s="10" t="n"/>
       <c r="B18" s="11" t="inlineStr">
         <is>
@@ -2332,50 +2116,17 @@
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>■ 將你的時空鎖鏈替換成腥紅特效。
-■ 將技能「時空鎖鏈」的特效替換為瓦爾時空先知。
-★ 1.5秒延遲後施加詛咒
-★ 詛咒無法套用至等級高於(0—20)的敵人
-★ 詛咒範圍為(1.5—3.1)公尺
-★ 詛咒會緩速目標(40—59)%
-★ 詛咒持續時間為(6—7.4)秒
-★ 詛咒使目標身上其他效果減緩25%失效
-★ base deal no damage 1
-★ can perform skill while moving 1
-▶ Blasphemy 光环诅咒之一</t>
+          <t>▶ Blasphemy 光环诅咒之一</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>■ 將技能「元素要害」的特效替換為深淵。
-■ 將技能「元素要害」的特效替換為幽暗碎魂。
-■ +8%的護甲值也會套用至元素傷害
-■ 能量護盾開始充能速度加快10%
-★ 1.5秒延遲後施加詛咒
-★ 詛咒無法套用至等級高於(0—20)的敵人
-★ 詛咒範圍為(1.5—3.1)公尺
-★ 詛咒使元素抗性(-59—-40)%
-★ 詛咒持續時間為(6—7.4)秒
-★ base deal no damage 1
-★ can perform skill while moving 1
-★ movement speed +% final while performing action -70
-▶ Blasphemy 降抗诅咒</t>
+          <t>▶ Blasphemy 降抗诅咒</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>■ 將你的衰弱替換成腥紅特效。
-■ 賦予技能: 招架
-■ 輕盾: 格擋時，會對敵人施加衰弱衰弱詛咒
-★ 1.5秒延遲後施加詛咒
-★ 詛咒無法套用至等級高於(0—20)的敵人
-★ 詛咒範圍為(1.5—3.1)公尺
-★ 詛咒使目標造成(20—29)%更少傷害
-★ 詛咒持續時間為(6—7.4)秒
-★ base deal no damage 1
-★ can perform skill while moving 1
-★ movement speed +% final while performing action -70
-▶ Blasphemy 减伤诅咒</t>
+          <t>▶ Blasphemy 减伤诅咒</t>
         </is>
       </c>
       <c r="F18" s="11" t="inlineStr">
@@ -2398,8 +2149,7 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>凋零光環
-(Level)
+          <t>Withering Presence
 Lv.18</t>
         </is>
       </c>
@@ -2415,14 +2165,11 @@
         </is>
       </c>
     </row>
-    <row r="21" outlineLevel="1" ht="92" customHeight="1">
+    <row r="21" outlineLevel="1" ht="76" customHeight="1">
       <c r="A21" s="10" t="n"/>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>★ 凋零持續時間為6秒
-★ 身處你存在範圍中的敵人每(1.42—1.8)秒承受凋零
-★ skill desired amount override 1
-▶ 凋零 debuff 叠层</t>
+          <t>▶ 凋零 debuff 叠层</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
@@ -2471,8 +2218,7 @@
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>脆弱
-(Level)
+          <t>Vulnerability
 Lv.19</t>
         </is>
       </c>
@@ -2502,20 +2248,11 @@
         </is>
       </c>
     </row>
-    <row r="26" outlineLevel="1" ht="140" customHeight="1">
+    <row r="26" outlineLevel="1" ht="36" customHeight="1">
       <c r="A26" s="10" t="n"/>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>■ 將你的脆弱替換成腥紅特效。
-★ 1.5秒延遲後施加詛咒
-★ 詛咒無法套用至等級高於(0—20)的敵人
-★ 詛咒範圍為(1.5—3.1)公尺
-★ 詛咒會減少(16—19210)總護甲
-★ 詛咒持續時間為(6—7.4)秒
-★ base deal no damage 1
-★ can perform skill while moving 1
-★ movement speed +% final while performing action -70
-▶ II 组手动诅咒（计入 Liminal 增伤）</t>
+          <t>▶ II 组手动诅咒（计入 Liminal 增伤）</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
@@ -2553,8 +2290,7 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>絕望
-(Level)
+          <t>Despair
 Lv.19</t>
         </is>
       </c>
@@ -2584,21 +2320,11 @@
         </is>
       </c>
     </row>
-    <row r="29" outlineLevel="1" ht="148" customHeight="1">
+    <row r="29" outlineLevel="1" ht="36" customHeight="1">
       <c r="A29" s="10" t="n"/>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>■ 將你的絕望替換成腥紅特效。
-■ 將你的絕望替換成譫妄特效。
-★ 1.5秒延遲後施加詛咒
-★ 詛咒無法套用至等級高於(0—20)的敵人
-★ 詛咒使混沌抗性(-49—-35)%
-★ 詛咒範圍為(1.5—3.1)公尺
-★ 詛咒持續時間為(6—7.4)秒
-★ base deal no damage 1
-★ can perform skill while moving 1
-★ movement speed +% final while performing action -70
-▶ II 组混沌诅咒</t>
+          <t>▶ II 组混沌诅咒</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Sync BD docs 2026-07-08-v1 (202607200344) from my-cloud-project@d60d7fc
</commit_message>
<xml_diff>
--- a/Coiling_Bolts_Blood_Mage_BD指南.xlsx
+++ b/Coiling_Bolts_Blood_Mage_BD指南.xlsx
@@ -404,9 +404,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>4</col>
       <colOff>0</colOff>
-      <row>17</row>
+      <row>11</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -429,9 +429,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>2</col>
+      <col>1</col>
       <colOff>0</colOff>
-      <row>20</row>
+      <row>14</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -456,7 +456,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>31</row>
+      <row>17</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -479,12 +479,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>2</col>
       <colOff>0</colOff>
-      <row>36</row>
+      <row>17</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="200025" cy="609600"/>
+    <ext cx="609600" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="9" name="Image 9" descr="Picture"/>
@@ -504,9 +504,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>3</col>
       <colOff>0</colOff>
-      <row>39</row>
+      <row>17</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -529,9 +529,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>4</col>
       <colOff>0</colOff>
-      <row>71</row>
+      <row>17</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -542,6 +542,206 @@
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId11"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId12"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="13" name="Image 13" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId13"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="14" name="Image 14" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId14"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>28</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId15"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>31</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="16" name="Image 16" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId16"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>36</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="200025" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId17"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>39</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="18" name="Image 18" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId18"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>71</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="19" name="Image 19" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId19"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1962,7 +2162,8 @@
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>Khatal's Rejuvenation</t>
+          <t>卡塔爾的恢復
+(Date)</t>
         </is>
       </c>
     </row>
@@ -1992,7 +2193,9 @@
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>▶ 生命痕跡族裔辅助</t>
+          <t>★ 被輔助技能所創造的痕跡會在拾取時賦予卡塔爾的回春
+★ base_cooldown_speed_+%
+▶ 生命痕跡族裔辅助</t>
         </is>
       </c>
     </row>
@@ -2005,7 +2208,8 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>Sigil of Power
+          <t>咒符之力
+(Level)
 Lv.18</t>
         </is>
       </c>
@@ -2030,11 +2234,20 @@
         </is>
       </c>
     </row>
-    <row r="15" outlineLevel="1" ht="36" customHeight="1">
+    <row r="15" outlineLevel="1" ht="140" customHeight="1">
       <c r="A15" s="10" t="n"/>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>▶ Boss 前铺设增伤法阵</t>
+          <t>■ 將技能「咒符之力」的特效替換為聖能。
+★ 疊層間至少1秒
+★ 符印範圍為3公尺
+★ 在區域中共消耗50%最大魔力時，獲得1個疊層
+★ 符印持續時間為(10—11.9)秒
+★ 疊層上限4
+★ 每層增益效果賦予(10—14)%更多法術傷害
+★ base number of sigil of power allowed 1
+★ can perform skill while moving 1
+▶ Boss 前铺设增伤法阵</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
@@ -2074,17 +2287,20 @@
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>Temporal Chains</t>
+          <t>時空鎖鏈
+(Level)</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>Elemental Weakness</t>
+          <t>元素要害
+(Level)</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>Enfeeble</t>
+          <t>衰弱
+(Level)</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
@@ -2098,7 +2314,7 @@
         </is>
       </c>
     </row>
-    <row r="18" outlineLevel="1" ht="140" customHeight="1">
+    <row r="18" outlineLevel="1" ht="164" customHeight="1">
       <c r="A18" s="10" t="n"/>
       <c r="B18" s="11" t="inlineStr">
         <is>
@@ -2116,17 +2332,50 @@
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>▶ Blasphemy 光环诅咒之一</t>
+          <t>■ 將你的時空鎖鏈替換成腥紅特效。
+■ 將技能「時空鎖鏈」的特效替換為瓦爾時空先知。
+★ 1.5秒延遲後施加詛咒
+★ 詛咒無法套用至等級高於(0—20)的敵人
+★ 詛咒範圍為(1.5—3.1)公尺
+★ 詛咒會緩速目標(40—59)%
+★ 詛咒持續時間為(6—7.4)秒
+★ 詛咒使目標身上其他效果減緩25%失效
+★ base deal no damage 1
+★ can perform skill while moving 1
+▶ Blasphemy 光环诅咒之一</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>▶ Blasphemy 降抗诅咒</t>
+          <t>■ 將技能「元素要害」的特效替換為深淵。
+■ 將技能「元素要害」的特效替換為幽暗碎魂。
+■ +8%的護甲值也會套用至元素傷害
+■ 能量護盾開始充能速度加快10%
+★ 1.5秒延遲後施加詛咒
+★ 詛咒無法套用至等級高於(0—20)的敵人
+★ 詛咒範圍為(1.5—3.1)公尺
+★ 詛咒使元素抗性(-59—-40)%
+★ 詛咒持續時間為(6—7.4)秒
+★ base deal no damage 1
+★ can perform skill while moving 1
+★ movement speed +% final while performing action -70
+▶ Blasphemy 降抗诅咒</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>▶ Blasphemy 减伤诅咒</t>
+          <t>■ 將你的衰弱替換成腥紅特效。
+■ 賦予技能: 招架
+■ 輕盾: 格擋時，會對敵人施加衰弱衰弱詛咒
+★ 1.5秒延遲後施加詛咒
+★ 詛咒無法套用至等級高於(0—20)的敵人
+★ 詛咒範圍為(1.5—3.1)公尺
+★ 詛咒使目標造成(20—29)%更少傷害
+★ 詛咒持續時間為(6—7.4)秒
+★ base deal no damage 1
+★ can perform skill while moving 1
+★ movement speed +% final while performing action -70
+▶ Blasphemy 减伤诅咒</t>
         </is>
       </c>
       <c r="F18" s="11" t="inlineStr">
@@ -2149,7 +2398,8 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Withering Presence
+          <t>凋零光環
+(Level)
 Lv.18</t>
         </is>
       </c>
@@ -2165,11 +2415,14 @@
         </is>
       </c>
     </row>
-    <row r="21" outlineLevel="1" ht="76" customHeight="1">
+    <row r="21" outlineLevel="1" ht="92" customHeight="1">
       <c r="A21" s="10" t="n"/>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>▶ 凋零 debuff 叠层</t>
+          <t>★ 凋零持續時間為6秒
+★ 身處你存在範圍中的敵人每(1.42—1.8)秒承受凋零
+★ skill desired amount override 1
+▶ 凋零 debuff 叠层</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
@@ -2218,7 +2471,8 @@
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>Vulnerability
+          <t>脆弱
+(Level)
 Lv.19</t>
         </is>
       </c>
@@ -2248,11 +2502,20 @@
         </is>
       </c>
     </row>
-    <row r="26" outlineLevel="1" ht="36" customHeight="1">
+    <row r="26" outlineLevel="1" ht="140" customHeight="1">
       <c r="A26" s="10" t="n"/>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>▶ II 组手动诅咒（计入 Liminal 增伤）</t>
+          <t>■ 將你的脆弱替換成腥紅特效。
+★ 1.5秒延遲後施加詛咒
+★ 詛咒無法套用至等級高於(0—20)的敵人
+★ 詛咒範圍為(1.5—3.1)公尺
+★ 詛咒會減少(16—19210)總護甲
+★ 詛咒持續時間為(6—7.4)秒
+★ base deal no damage 1
+★ can perform skill while moving 1
+★ movement speed +% final while performing action -70
+▶ II 组手动诅咒（计入 Liminal 增伤）</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
@@ -2290,7 +2553,8 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Despair
+          <t>絕望
+(Level)
 Lv.19</t>
         </is>
       </c>
@@ -2320,11 +2584,21 @@
         </is>
       </c>
     </row>
-    <row r="29" outlineLevel="1" ht="36" customHeight="1">
+    <row r="29" outlineLevel="1" ht="148" customHeight="1">
       <c r="A29" s="10" t="n"/>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>▶ II 组混沌诅咒</t>
+          <t>■ 將你的絕望替換成腥紅特效。
+■ 將你的絕望替換成譫妄特效。
+★ 1.5秒延遲後施加詛咒
+★ 詛咒無法套用至等級高於(0—20)的敵人
+★ 詛咒使混沌抗性(-49—-35)%
+★ 詛咒範圍為(1.5—3.1)公尺
+★ 詛咒持續時間為(6—7.4)秒
+★ base deal no damage 1
+★ can perform skill while moving 1
+★ movement speed +% final while performing action -70
+▶ II 组混沌诅咒</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Sync BD docs 2026-07-08-v1 (202607200717) from my-cloud-project@7546c42
</commit_message>
<xml_diff>
--- a/Coiling_Bolts_Blood_Mage_BD指南.xlsx
+++ b/Coiling_Bolts_Blood_Mage_BD指南.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00-目录" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01-机制" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02-武器组" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03-天赋" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04-常见问题" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="00-目录" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="01-机制" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="02-武器组" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="03-天赋" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="04-常见问题" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -276,7 +276,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>1</col>
@@ -291,13 +291,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -316,13 +316,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -341,13 +341,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -366,13 +366,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -391,13 +391,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -416,13 +416,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId6"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -441,13 +441,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId7"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -466,13 +466,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId8"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId8"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -491,13 +491,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId9"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId9"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -516,13 +516,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId10"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId10"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -541,13 +541,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId11"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId11"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -566,13 +566,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId12"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId12"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -591,13 +591,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId13"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId13"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -616,13 +616,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId14"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId14"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -641,13 +641,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId15"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId15"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -666,13 +666,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId16"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId16"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -691,13 +691,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId17"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId17"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -716,13 +716,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId18"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId18"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -741,13 +741,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId19"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId19"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2742,9 +2742,9 @@
 ★ 你施加的詛咒無視詛咒上限
 ★ 目標每受一個詛咒影響，法術擊中即獲得(23—31)%傷害的額外混沌傷害
 ★ 目標每受一個詛咒影響，法術擊中即獲得(23—31)%傷害的額外物理傷害
-「In that moment, Viridi's bones became 
-branches, weaving over the Darkness. 
-She coiled around the nothing, 
+「In that moment, Viridi's bones became 
+branches, weaving over the Darkness. 
+She coiled around the nothing, 
 trapping it within her everything.」
 ▶ BD 用途：BD 核心：赋予寂缠弹；诅咒幅度归零但无视诅咒上限，每诅咒巨额额外物理/混沌
 🔗 https://poe2db.tw/tw/Liminal_Coil
@@ -2779,8 +2779,8 @@
 ★ +100精魂
 ★ +(50—75)%冰冷抗性
 ★ 存在範圍的範圍加倍
-「Nature respects the strong
-And paints the snow red
+「Nature respects the strong
+And paints the snow red
 With the blood of the weak」
 ▶ BD 用途：+100 Spirit，Blasphemy 多诅咒必备
 🔗 https://poe2db.tw/tw/Alphas_Howl
@@ -3056,7 +3056,7 @@
 ★ +10點智慧
 ★ +(7—13)%混沌抗性
 ★ 以法術暴擊時，施加(1—3)層的暴擊弱點
-「The horrors we imagined as children
+「The horrors we imagined as children
 still exist somewhere in the dark...」
 ▶ BD 用途：II 组副手：法术暴击叠 Critical Weakness
 🔗 https://poe2db.tw/tw/Effigy_of_Cruelty

</xml_diff>

<commit_message>
Sync BD docs 2026-07-08-v1 (202607200721) from my-cloud-project@05c8b38
</commit_message>
<xml_diff>
--- a/Coiling_Bolts_Blood_Mage_BD指南.xlsx
+++ b/Coiling_Bolts_Blood_Mage_BD指南.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="00-目录" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="01-机制" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="02-武器组" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="03-天赋" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="04-常见问题" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00-目录" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01-机制" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02-武器组" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03-天赋" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04-常见问题" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -276,7 +276,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>1</col>
@@ -291,13 +291,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -316,13 +316,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -341,13 +341,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId3"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -366,13 +366,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId4"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -391,13 +391,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId5"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -416,13 +416,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId6"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -441,13 +441,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId7"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -466,13 +466,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId8"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId8"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -491,13 +491,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId9"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId9"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -516,13 +516,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId10"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId10"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -541,13 +541,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId11"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId11"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -566,13 +566,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId12"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId12"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -591,13 +591,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId13"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId13"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -616,13 +616,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId14"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId14"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -641,13 +641,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId15"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId15"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -666,13 +666,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId16"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId16"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -691,13 +691,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId17"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId17"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -716,13 +716,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId18"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId18"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -741,13 +741,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId19"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId19"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2742,9 +2742,9 @@
 ★ 你施加的詛咒無視詛咒上限
 ★ 目標每受一個詛咒影響，法術擊中即獲得(23—31)%傷害的額外混沌傷害
 ★ 目標每受一個詛咒影響，法術擊中即獲得(23—31)%傷害的額外物理傷害
-「In that moment, Viridi's bones became 
-branches, weaving over the Darkness. 
-She coiled around the nothing, 
+「In that moment, Viridi's bones became 
+branches, weaving over the Darkness. 
+She coiled around the nothing, 
 trapping it within her everything.」
 ▶ BD 用途：BD 核心：赋予寂缠弹；诅咒幅度归零但无视诅咒上限，每诅咒巨额额外物理/混沌
 🔗 https://poe2db.tw/tw/Liminal_Coil
@@ -2779,8 +2779,8 @@
 ★ +100精魂
 ★ +(50—75)%冰冷抗性
 ★ 存在範圍的範圍加倍
-「Nature respects the strong
-And paints the snow red
+「Nature respects the strong
+And paints the snow red
 With the blood of the weak」
 ▶ BD 用途：+100 Spirit，Blasphemy 多诅咒必备
 🔗 https://poe2db.tw/tw/Alphas_Howl
@@ -3056,7 +3056,7 @@
 ★ +10點智慧
 ★ +(7—13)%混沌抗性
 ★ 以法術暴擊時，施加(1—3)層的暴擊弱點
-「The horrors we imagined as children
+「The horrors we imagined as children
 still exist somewhere in the dark...」
 ▶ BD 用途：II 组副手：法术暴击叠 Critical Weakness
 🔗 https://poe2db.tw/tw/Effigy_of_Cruelty

</xml_diff>